<commit_message>
Complete Test management and Testing
</commit_message>
<xml_diff>
--- a/Test - Dev_person4-test.xlsx
+++ b/Test - Dev_person4-test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3A66EEBB-8280-4910-A094-14E4B581864C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3634A47D-799C-4E8C-9802-57FF5B27302C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="34">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -37,16 +37,7 @@
     <t>Expected Result</t>
   </si>
   <si>
-    <t>Actual Result</t>
-  </si>
-  <si>
-    <t>Status</t>
-  </si>
-  <si>
     <t>TC01</t>
-  </si>
-  <si>
-    <t>Pass</t>
   </si>
   <si>
     <t>TC02</t>
@@ -172,7 +163,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -184,8 +175,14 @@
         <fgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -208,20 +205,116 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -536,166 +629,138 @@
     <col min="7" max="7" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:7" s="13" customFormat="1" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
     </row>
     <row r="2" spans="1:7" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>8</v>
-      </c>
+      <c r="A2" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="E2" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F2" s="5"/>
+      <c r="G2" s="6"/>
     </row>
     <row r="3" spans="1:7" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>8</v>
-      </c>
+      <c r="A3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="E3" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="F3" s="5"/>
+      <c r="G3" s="6"/>
     </row>
     <row r="4" spans="1:7" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>24</v>
+      <c r="A4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>21</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>8</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="F4" s="5"/>
+      <c r="G4" s="6"/>
     </row>
     <row r="5" spans="1:7" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>25</v>
+      <c r="A5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>22</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>8</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="F5" s="5"/>
+      <c r="G5" s="6"/>
     </row>
     <row r="6" spans="1:7" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>26</v>
+      <c r="A6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>23</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>8</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="F6" s="5"/>
+      <c r="G6" s="6"/>
     </row>
     <row r="7" spans="1:7" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>30</v>
+      <c r="A7" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>8</v>
-      </c>
+        <v>29</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="F7" s="5"/>
+      <c r="G7" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>